<commit_message>
Routing and LCSC BOM of Both boards
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Altiumgenerated_Control_Board.xlsx
+++ b/Deliverables/BOM/Altiumgenerated_Control_Board.xlsx
@@ -4,20 +4,20 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24000" windowHeight="9795"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Altiumgenerated_Control_Board" sheetId="1" r:id="rId1"/>
+    <sheet name="Free Documents" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Altiumgenerated_Control_Board!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Free Documents'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="123">
   <si>
     <t>Comment</t>
   </si>
@@ -64,7 +64,7 @@
     <t>CAP CER 0.1UF 100V X7R 0603</t>
   </si>
   <si>
-    <t>C2, C4, C6, C7, C8, C9, C10, C11, C12, C13, C14, C15, C16, C20, C21, C22, C23, C24, C25, C30, C31, C41</t>
+    <t>C2, C4, C6, C7, C8, C9, C10, C11, C12, C13, C14, C15, C16, C20, C21, C22, C23, C24, C25, C30, C31, C34, C35, C41</t>
   </si>
   <si>
     <t>Cap0603</t>
@@ -187,7 +187,7 @@
     <t>Green 520~535nm 0402 Light Emitting Diodes (LED) RoHS</t>
   </si>
   <si>
-    <t>LED1, LED2</t>
+    <t>LED1, LED2, LED3</t>
   </si>
   <si>
     <t>LED 0402</t>
@@ -214,7 +214,7 @@
     <t>RES SMD 10K OHM 5% 1/10W 0603</t>
   </si>
   <si>
-    <t>R1, R2, R3, R4, R5, R9, R14, R15, R16, R23, R24, R41, R42</t>
+    <t>R1, R2, R3, R4, R5, R9, R14, R15, R16, R23, R41, R42</t>
   </si>
   <si>
     <t>Res0603</t>
@@ -253,7 +253,7 @@
     <t>RES SMD 1K OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>R8, R10, R40</t>
+    <t>R8, R10, R17, R40</t>
   </si>
   <si>
     <t>RC0603FR-071KL</t>
@@ -271,6 +271,30 @@
     <t>RT0603CRD0712K1L</t>
   </si>
   <si>
+    <t>100R</t>
+  </si>
+  <si>
+    <t>RES SMD 100 OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>R18, R19</t>
+  </si>
+  <si>
+    <t>RC0603FR-07100RL</t>
+  </si>
+  <si>
+    <t>470R</t>
+  </si>
+  <si>
+    <t>RES SMD 470 OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>R20</t>
+  </si>
+  <si>
+    <t>RC0603FR-07470RL</t>
+  </si>
+  <si>
     <t>Solder Bridge</t>
   </si>
   <si>
@@ -316,6 +340,18 @@
     <t>ON Semiconductor</t>
   </si>
   <si>
+    <t>TXB0102DCUT</t>
+  </si>
+  <si>
+    <t>IC TRNSLTR BIDIRECTIONAL US8</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
     <t>TLE5012BE5000FUMA1</t>
   </si>
   <si>
@@ -326,18 +362,6 @@
   </si>
   <si>
     <t>Infineon</t>
-  </si>
-  <si>
-    <t>SN74LVCH8T245PWR</t>
-  </si>
-  <si>
-    <t>IC TRANSLATION TXRX 5.5V 24TSSOP</t>
-  </si>
-  <si>
-    <t>U5</t>
-  </si>
-  <si>
-    <t>Texas Instruments</t>
   </si>
   <si>
     <t>C3E-25.000-8-1015-X-M</t>
@@ -369,10 +393,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -380,6 +404,43 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -391,17 +452,30 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -416,38 +490,10 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -461,30 +507,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -499,23 +529,17 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color theme="3"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -542,31 +566,121 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -578,7 +692,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -590,31 +716,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -626,78 +734,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -705,18 +741,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -925,35 +949,26 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -974,6 +989,21 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
       <right style="thin">
@@ -988,17 +1018,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1018,15 +1042,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1036,130 +1060,130 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1554,7 +1578,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="6" width="19.6761904761905" customWidth="1"/>
@@ -1607,7 +1631,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" ht="75" spans="1:7">
+    <row r="3" ht="90" spans="1:7">
       <c r="A3" s="17" t="s">
         <v>13</v>
       </c>
@@ -1624,7 +1648,7 @@
         <v>17</v>
       </c>
       <c r="F3" s="9">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G3" s="19" t="s">
         <v>18</v>
@@ -1831,7 +1855,7 @@
         <v>54</v>
       </c>
       <c r="F12" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" s="19" t="s">
         <v>58</v>
@@ -1875,7 +1899,7 @@
         <v>67</v>
       </c>
       <c r="F14" s="9">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G14" s="19" t="s">
         <v>18</v>
@@ -1944,7 +1968,7 @@
         <v>79</v>
       </c>
       <c r="F17" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G17" s="19" t="s">
         <v>18</v>
@@ -1984,61 +2008,61 @@
         <v>86</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F19" s="9">
-        <v>5</v>
-      </c>
-      <c r="G19" s="10"/>
+        <v>2</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="20" ht="30" spans="1:7">
       <c r="A20" s="17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F20" s="9">
         <v>1</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>90</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" ht="30" spans="1:7">
       <c r="A21" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B21" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>91</v>
-      </c>
       <c r="E21" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F21" s="9">
-        <v>1</v>
-      </c>
-      <c r="G21" s="19" t="s">
-        <v>94</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G21" s="10"/>
     </row>
     <row r="22" ht="30" spans="1:7">
       <c r="A22" s="17" t="s">
@@ -2132,27 +2156,73 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" ht="45" spans="1:7">
-      <c r="A26" s="20" t="s">
+    <row r="26" ht="30" spans="1:7">
+      <c r="A26" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E26" s="21" t="s">
+      <c r="E26" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="F26" s="12">
+      <c r="F26" s="9">
         <v>1</v>
       </c>
-      <c r="G26" s="22" t="s">
+      <c r="G26" s="19" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="27" ht="30" spans="1:7">
+      <c r="A27" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" s="9">
+        <v>1</v>
+      </c>
+      <c r="G27" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="28" ht="45" spans="1:7">
+      <c r="A28" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="F28" s="12">
+        <v>1</v>
+      </c>
+      <c r="G28" s="22" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>